<commit_message>
Added grids to divertingunits.xslx.
</commit_message>
<xml_diff>
--- a/example_data/other_units/divertingunits.xlsx
+++ b/example_data/other_units/divertingunits.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
@@ -20,15 +20,24 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t xml:space="preserve">name</t>
   </si>
   <si>
+    <t xml:space="preserve">inputgrid</t>
+  </si>
+  <si>
     <t xml:space="preserve">inputnode</t>
   </si>
   <si>
+    <t xml:space="preserve">outputgrid</t>
+  </si>
+  <si>
     <t xml:space="preserve">outputnode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">divertinggrid</t>
   </si>
   <si>
     <t xml:space="preserve">divertingnode</t>
@@ -347,7 +356,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20.81"/>
@@ -355,9 +364,12 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="15.51"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="16.8"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="15.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="19.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="13.75"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="23.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -370,14 +382,23 @@
       <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>